<commit_message>
Fill Crop Efficiency acreage, drop cost-per-ton chart and detail table
</commit_message>
<xml_diff>
--- a/data/Crop Efficiency - Stat Cards.xlsx
+++ b/data/Crop Efficiency - Stat Cards.xlsx
@@ -459,6 +459,12 @@
           <t>owned &amp; rented</t>
         </is>
       </c>
+      <c r="C2" t="n">
+        <v>2500</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2500</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">

</xml_diff>

<commit_message>
Add Wheat/Rye yield stat card, fill MI averages for crop yields, add data-sources appendix
</commit_message>
<xml_diff>
--- a/data/Crop Efficiency - Stat Cards.xlsx
+++ b/data/Crop Efficiency - Stat Cards.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -502,6 +502,18 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Wheat/Rye Yield</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>bu/acre, vs. MI avg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Total Value of Crops Produced stat card to Crop Efficiency
$1,413,060 = wheat (200 ac x 60 bu/ac x $6.28/bu, real 2023 Michigan
NASS price) + alfalfa (700 ac x 9.8 T/ac x $195.00/ton, using the 2023
Michigan dry alfalfa hay price as an approximation for silage, per
request). Corn silage is excluded and called out on the card itself:
NASS reports Michigan corn-silage production but never publishes a
price for it, so this total only covers 900 of 2,500 acres (36%), not
full-farm crop value. Full math in footnote 2 in the Appendix.

Also fix "below avg" -> "below MI avg" on the yield stat card deltas,
add a .stats-6 grid variant for the now 6-card row, and sync
data/Crop Efficiency - Stat Cards.xlsx.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Crop Efficiency - Stat Cards.xlsx
+++ b/data/Crop Efficiency - Stat Cards.xlsx
@@ -523,7 +523,21 @@
         <v>60</v>
       </c>
     </row>
-    <row r="7"/>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Total Value of Crops Produced</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>wheat + alfalfa only, excl. corn silage</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1413060</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>